<commit_message>
feat: replace sheetjs by excelj & implement 1st-class stream support
</commit_message>
<xml_diff>
--- a/examples/financial-report.xlsx
+++ b/examples/financial-report.xlsx
@@ -32,7 +32,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="12">
+  <numFmts count="10">
     <numFmt numFmtId="165" formatCode="MMM YYYY"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
@@ -43,10 +43,8 @@
     <numFmt numFmtId="172" formatCode="$#,##0.00"/>
     <numFmt numFmtId="173" formatCode="$#,##0.00"/>
     <numFmt numFmtId="174" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="175" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="176" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -88,37 +86,12 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF0000"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF0000"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF0000"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF0000"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
       <color rgb="007500"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <color rgb="007500"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF0000"/>
     </font>
     <font>
       <sz val="11"/>
@@ -184,7 +157,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -494,7 +467,7 @@
       <top style="thin">
         <color rgb="000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color rgb="000000"/>
       </bottom>
       <diagonal/>
@@ -509,82 +482,7 @@
       <top style="thin">
         <color rgb="000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="000000"/>
-      </top>
       <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thin">
         <color rgb="000000"/>
       </bottom>
       <diagonal/>
@@ -638,7 +536,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -705,28 +603,13 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="17" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="18" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="13" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="14" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1109,34 +992,34 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="4" t="str">
-        <v>2023-05</v>
+        <v>2023-10</v>
       </c>
       <c r="B2" s="5" t="str">
-        <v>Human Resources</v>
+        <v>Customer Support</v>
       </c>
       <c r="C2" s="6">
-        <v>80336</v>
+        <v>75123</v>
       </c>
       <c r="D2" s="6">
-        <v>21916</v>
+        <v>20926</v>
       </c>
       <c r="E2" s="7">
-        <v>58420</v>
+        <v>54197</v>
       </c>
       <c r="F2" s="8" t="str">
-        <v>72.72%</v>
+        <v>72.14%</v>
       </c>
       <c r="G2" s="6">
-        <v>194223</v>
+        <v>158871</v>
       </c>
       <c r="H2" s="6">
-        <v>56200</v>
+        <v>86095</v>
       </c>
       <c r="I2" s="7">
-        <v>138023</v>
+        <v>72776</v>
       </c>
       <c r="J2" s="9">
-        <v>32.72666666666667</v>
+        <v>37.83</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -1144,19 +1027,19 @@
         <v/>
       </c>
       <c r="B3" s="11" t="str">
-        <v>Sales</v>
+        <v>Customer Support</v>
       </c>
       <c r="C3" s="12">
-        <v>97976</v>
+        <v>20752</v>
       </c>
       <c r="D3" s="12">
-        <v>7774</v>
+        <v>17084</v>
       </c>
       <c r="E3" s="13">
-        <v>90202</v>
+        <v>3668</v>
       </c>
       <c r="F3" s="14" t="str">
-        <v>92.07%</v>
+        <v>17.68%</v>
       </c>
       <c r="G3" s="11" t="str">
         <v/>
@@ -1176,19 +1059,19 @@
         <v/>
       </c>
       <c r="B4" s="17" t="str">
-        <v>Customer Support</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C4" s="18">
-        <v>15911</v>
+        <v>62996</v>
       </c>
       <c r="D4" s="18">
-        <v>26510</v>
+        <v>48085</v>
       </c>
       <c r="E4" s="19">
-        <v>-10599</v>
+        <v>14911</v>
       </c>
       <c r="F4" s="20" t="str">
-        <v>-66.61%</v>
+        <v>23.67%</v>
       </c>
       <c r="G4" s="17" t="str">
         <v/>
@@ -1205,34 +1088,34 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="str">
-        <v>2023-05</v>
+        <v>2023-03</v>
       </c>
       <c r="B5" s="5" t="str">
-        <v>Sales</v>
+        <v>Human Resources</v>
       </c>
       <c r="C5" s="6">
-        <v>64442</v>
+        <v>42667</v>
       </c>
       <c r="D5" s="6">
-        <v>38483</v>
+        <v>10024</v>
       </c>
       <c r="E5" s="7">
-        <v>25959</v>
+        <v>32643</v>
       </c>
       <c r="F5" s="8" t="str">
-        <v>40.28%</v>
+        <v>76.51%</v>
       </c>
       <c r="G5" s="6">
-        <v>145047</v>
+        <v>143580</v>
       </c>
       <c r="H5" s="6">
-        <v>118052</v>
+        <v>94408</v>
       </c>
       <c r="I5" s="7">
-        <v>26995</v>
+        <v>49172</v>
       </c>
       <c r="J5" s="9">
-        <v>14.256666666666668</v>
+        <v>35.513333333333335</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -1240,19 +1123,19 @@
         <v/>
       </c>
       <c r="B6" s="11" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="C6" s="12">
-        <v>39864</v>
+        <v>56344</v>
       </c>
       <c r="D6" s="12">
-        <v>40866</v>
-      </c>
-      <c r="E6" s="22">
-        <v>-1002</v>
-      </c>
-      <c r="F6" s="23" t="str">
-        <v>-2.51%</v>
+        <v>41280</v>
+      </c>
+      <c r="E6" s="13">
+        <v>15064</v>
+      </c>
+      <c r="F6" s="14" t="str">
+        <v>26.74%</v>
       </c>
       <c r="G6" s="11" t="str">
         <v/>
@@ -1272,19 +1155,19 @@
         <v/>
       </c>
       <c r="B7" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Human Resources</v>
       </c>
       <c r="C7" s="18">
-        <v>40741</v>
+        <v>44569</v>
       </c>
       <c r="D7" s="18">
-        <v>38703</v>
-      </c>
-      <c r="E7" s="24">
-        <v>2038</v>
-      </c>
-      <c r="F7" s="25" t="str">
-        <v>5%</v>
+        <v>43104</v>
+      </c>
+      <c r="E7" s="19">
+        <v>1465</v>
+      </c>
+      <c r="F7" s="20" t="str">
+        <v>3.29%</v>
       </c>
       <c r="G7" s="17" t="str">
         <v/>
@@ -1301,34 +1184,34 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="str">
-        <v>2023-12</v>
+        <v>2023-06</v>
       </c>
       <c r="B8" s="5" t="str">
-        <v>R&amp;D</v>
+        <v>Human Resources</v>
       </c>
       <c r="C8" s="6">
-        <v>76606</v>
+        <v>59635</v>
       </c>
       <c r="D8" s="6">
-        <v>47128</v>
+        <v>25739</v>
       </c>
       <c r="E8" s="7">
-        <v>29478</v>
+        <v>33896</v>
       </c>
       <c r="F8" s="8" t="str">
-        <v>38.48%</v>
+        <v>56.84%</v>
       </c>
       <c r="G8" s="6">
-        <v>195532</v>
+        <v>252115</v>
       </c>
       <c r="H8" s="6">
-        <v>101061</v>
+        <v>117520</v>
       </c>
       <c r="I8" s="7">
-        <v>94471</v>
+        <v>134595</v>
       </c>
       <c r="J8" s="9">
-        <v>49.423333333333325</v>
+        <v>53.75333333333333</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -1336,19 +1219,19 @@
         <v/>
       </c>
       <c r="B9" s="11" t="str">
-        <v>Customer Support</v>
+        <v>Sales</v>
       </c>
       <c r="C9" s="12">
-        <v>62937</v>
+        <v>93467</v>
       </c>
       <c r="D9" s="12">
-        <v>31017</v>
+        <v>48184</v>
       </c>
       <c r="E9" s="13">
-        <v>31920</v>
+        <v>45283</v>
       </c>
       <c r="F9" s="14" t="str">
-        <v>50.72%</v>
+        <v>48.45%</v>
       </c>
       <c r="G9" s="11" t="str">
         <v/>
@@ -1371,16 +1254,16 @@
         <v>Sales</v>
       </c>
       <c r="C10" s="18">
-        <v>55989</v>
+        <v>99013</v>
       </c>
       <c r="D10" s="18">
-        <v>22916</v>
-      </c>
-      <c r="E10" s="24">
-        <v>33073</v>
-      </c>
-      <c r="F10" s="25" t="str">
-        <v>59.07%</v>
+        <v>43597</v>
+      </c>
+      <c r="E10" s="19">
+        <v>55416</v>
+      </c>
+      <c r="F10" s="20" t="str">
+        <v>55.97%</v>
       </c>
       <c r="G10" s="17" t="str">
         <v/>
@@ -1397,34 +1280,34 @@
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="str">
-        <v>2023-09</v>
+        <v>2023-12</v>
       </c>
       <c r="B11" s="5" t="str">
-        <v>Customer Support</v>
+        <v>Human Resources</v>
       </c>
       <c r="C11" s="6">
-        <v>59106</v>
+        <v>69443</v>
       </c>
       <c r="D11" s="6">
-        <v>41396</v>
+        <v>43038</v>
       </c>
       <c r="E11" s="7">
-        <v>17710</v>
+        <v>26405</v>
       </c>
       <c r="F11" s="8" t="str">
-        <v>29.96%</v>
+        <v>38.02%</v>
       </c>
       <c r="G11" s="6">
-        <v>168847</v>
+        <v>153944</v>
       </c>
       <c r="H11" s="6">
-        <v>63633</v>
+        <v>83220</v>
       </c>
       <c r="I11" s="7">
-        <v>105214</v>
+        <v>70724</v>
       </c>
       <c r="J11" s="9">
-        <v>62.330000000000005</v>
+        <v>34.59</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -1432,19 +1315,19 @@
         <v/>
       </c>
       <c r="B12" s="11" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="C12" s="12">
-        <v>47440</v>
+        <v>62410</v>
       </c>
       <c r="D12" s="12">
-        <v>14469</v>
+        <v>16290</v>
       </c>
       <c r="E12" s="13">
-        <v>32971</v>
+        <v>46120</v>
       </c>
       <c r="F12" s="14" t="str">
-        <v>69.5%</v>
+        <v>73.9%</v>
       </c>
       <c r="G12" s="11" t="str">
         <v/>
@@ -1464,19 +1347,19 @@
         <v/>
       </c>
       <c r="B13" s="17" t="str">
-        <v>Human Resources</v>
+        <v>Marketing</v>
       </c>
       <c r="C13" s="18">
-        <v>62301</v>
+        <v>22091</v>
       </c>
       <c r="D13" s="18">
-        <v>7768</v>
-      </c>
-      <c r="E13" s="24">
-        <v>54533</v>
-      </c>
-      <c r="F13" s="25" t="str">
-        <v>87.53%</v>
+        <v>23892</v>
+      </c>
+      <c r="E13" s="22">
+        <v>-1801</v>
+      </c>
+      <c r="F13" s="23" t="str">
+        <v>-8.15%</v>
       </c>
       <c r="G13" s="17" t="str">
         <v/>
@@ -1493,34 +1376,34 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="str">
-        <v>2023-09</v>
+        <v>2023-03</v>
       </c>
       <c r="B14" s="5" t="str">
-        <v>Sales</v>
+        <v>Marketing</v>
       </c>
       <c r="C14" s="6">
-        <v>69580</v>
+        <v>58907</v>
       </c>
       <c r="D14" s="6">
-        <v>16886</v>
+        <v>14681</v>
       </c>
       <c r="E14" s="7">
-        <v>52694</v>
+        <v>44226</v>
       </c>
       <c r="F14" s="8" t="str">
-        <v>75.73%</v>
+        <v>75.08%</v>
       </c>
       <c r="G14" s="6">
-        <v>232648</v>
+        <v>105805</v>
       </c>
       <c r="H14" s="6">
-        <v>83522</v>
+        <v>47122</v>
       </c>
       <c r="I14" s="7">
-        <v>149126</v>
+        <v>58683</v>
       </c>
       <c r="J14" s="9">
-        <v>63.95666666666667</v>
+        <v>44.96333333333333</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -1528,19 +1411,19 @@
         <v/>
       </c>
       <c r="B15" s="11" t="str">
-        <v>Human Resources</v>
+        <v>Customer Support</v>
       </c>
       <c r="C15" s="12">
-        <v>70895</v>
+        <v>24859</v>
       </c>
       <c r="D15" s="12">
-        <v>35495</v>
+        <v>13627</v>
       </c>
       <c r="E15" s="13">
-        <v>35400</v>
+        <v>11232</v>
       </c>
       <c r="F15" s="14" t="str">
-        <v>49.93%</v>
+        <v>45.18%</v>
       </c>
       <c r="G15" s="11" t="str">
         <v/>
@@ -1560,19 +1443,19 @@
         <v/>
       </c>
       <c r="B16" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Customer Support</v>
       </c>
       <c r="C16" s="18">
-        <v>92173</v>
+        <v>22039</v>
       </c>
       <c r="D16" s="18">
-        <v>31141</v>
-      </c>
-      <c r="E16" s="24">
-        <v>61032</v>
-      </c>
-      <c r="F16" s="25" t="str">
-        <v>66.21%</v>
+        <v>18814</v>
+      </c>
+      <c r="E16" s="19">
+        <v>3225</v>
+      </c>
+      <c r="F16" s="20" t="str">
+        <v>14.63%</v>
       </c>
       <c r="G16" s="17" t="str">
         <v/>
@@ -1589,34 +1472,34 @@
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="str">
-        <v>2023-09</v>
+        <v>2023-12</v>
       </c>
       <c r="B17" s="5" t="str">
         <v>R&amp;D</v>
       </c>
       <c r="C17" s="6">
-        <v>34994</v>
+        <v>75289</v>
       </c>
       <c r="D17" s="6">
-        <v>6620</v>
+        <v>39784</v>
       </c>
       <c r="E17" s="7">
-        <v>28374</v>
+        <v>35505</v>
       </c>
       <c r="F17" s="8" t="str">
-        <v>81.08%</v>
+        <v>47.16%</v>
       </c>
       <c r="G17" s="6">
-        <v>153497</v>
+        <v>161258</v>
       </c>
       <c r="H17" s="6">
-        <v>61087</v>
+        <v>118258</v>
       </c>
       <c r="I17" s="7">
-        <v>92410</v>
+        <v>43000</v>
       </c>
       <c r="J17" s="9">
-        <v>48.49</v>
+        <v>15.86</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -1624,19 +1507,19 @@
         <v/>
       </c>
       <c r="B18" s="11" t="str">
-        <v>R&amp;D</v>
+        <v>Customer Support</v>
       </c>
       <c r="C18" s="12">
-        <v>36233</v>
+        <v>58928</v>
       </c>
       <c r="D18" s="12">
-        <v>44935</v>
-      </c>
-      <c r="E18" s="22">
-        <v>-8702</v>
-      </c>
-      <c r="F18" s="23" t="str">
-        <v>-24.02%</v>
+        <v>45290</v>
+      </c>
+      <c r="E18" s="13">
+        <v>13638</v>
+      </c>
+      <c r="F18" s="14" t="str">
+        <v>23.14%</v>
       </c>
       <c r="G18" s="11" t="str">
         <v/>
@@ -1656,19 +1539,19 @@
         <v/>
       </c>
       <c r="B19" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Marketing</v>
       </c>
       <c r="C19" s="18">
-        <v>82270</v>
+        <v>27041</v>
       </c>
       <c r="D19" s="18">
-        <v>9532</v>
-      </c>
-      <c r="E19" s="24">
-        <v>72738</v>
-      </c>
-      <c r="F19" s="25" t="str">
-        <v>88.41%</v>
+        <v>33184</v>
+      </c>
+      <c r="E19" s="22">
+        <v>-6143</v>
+      </c>
+      <c r="F19" s="23" t="str">
+        <v>-22.72%</v>
       </c>
       <c r="G19" s="17" t="str">
         <v/>
@@ -1685,34 +1568,34 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="str">
-        <v>2023-06</v>
+        <v>2023-07</v>
       </c>
       <c r="B20" s="5" t="str">
-        <v>Human Resources</v>
+        <v>Sales</v>
       </c>
       <c r="C20" s="6">
-        <v>97059</v>
+        <v>40407</v>
       </c>
       <c r="D20" s="6">
-        <v>49907</v>
+        <v>31604</v>
       </c>
       <c r="E20" s="7">
-        <v>47152</v>
+        <v>8803</v>
       </c>
       <c r="F20" s="8" t="str">
-        <v>48.58%</v>
+        <v>21.79%</v>
       </c>
       <c r="G20" s="6">
-        <v>220262</v>
+        <v>196964</v>
       </c>
       <c r="H20" s="6">
-        <v>94758</v>
+        <v>88282</v>
       </c>
       <c r="I20" s="7">
-        <v>125504</v>
+        <v>108682</v>
       </c>
       <c r="J20" s="9">
-        <v>42.98666666666666</v>
+        <v>49.48666666666666</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1720,19 +1603,19 @@
         <v/>
       </c>
       <c r="B21" s="11" t="str">
-        <v>Marketing</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C21" s="12">
-        <v>88717</v>
+        <v>87221</v>
       </c>
       <c r="D21" s="12">
-        <v>5884</v>
+        <v>28428</v>
       </c>
       <c r="E21" s="13">
-        <v>82833</v>
+        <v>58793</v>
       </c>
       <c r="F21" s="14" t="str">
-        <v>93.37%</v>
+        <v>67.41%</v>
       </c>
       <c r="G21" s="11" t="str">
         <v/>
@@ -1752,19 +1635,19 @@
         <v/>
       </c>
       <c r="B22" s="17" t="str">
-        <v>Sales</v>
+        <v>Human Resources</v>
       </c>
       <c r="C22" s="18">
-        <v>34486</v>
+        <v>69336</v>
       </c>
       <c r="D22" s="18">
-        <v>38967</v>
+        <v>28250</v>
       </c>
       <c r="E22" s="19">
-        <v>-4481</v>
+        <v>41086</v>
       </c>
       <c r="F22" s="20" t="str">
-        <v>-12.99%</v>
+        <v>59.26%</v>
       </c>
       <c r="G22" s="17" t="str">
         <v/>
@@ -1781,34 +1664,34 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="str">
-        <v>2023-12</v>
+        <v>2023-08</v>
       </c>
       <c r="B23" s="5" t="str">
-        <v>Marketing</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C23" s="6">
-        <v>84827</v>
+        <v>38694</v>
       </c>
       <c r="D23" s="6">
-        <v>46709</v>
+        <v>35282</v>
       </c>
       <c r="E23" s="7">
-        <v>38118</v>
+        <v>3412</v>
       </c>
       <c r="F23" s="8" t="str">
-        <v>44.94%</v>
+        <v>8.82%</v>
       </c>
       <c r="G23" s="6">
-        <v>203207</v>
+        <v>166132</v>
       </c>
       <c r="H23" s="6">
-        <v>109645</v>
+        <v>101684</v>
       </c>
       <c r="I23" s="7">
-        <v>93562</v>
+        <v>64448</v>
       </c>
       <c r="J23" s="9">
-        <v>26.52333333333333</v>
+        <v>35.06</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
@@ -1819,16 +1702,16 @@
         <v>Customer Support</v>
       </c>
       <c r="C24" s="12">
-        <v>25011</v>
+        <v>59853</v>
       </c>
       <c r="D24" s="12">
-        <v>33468</v>
-      </c>
-      <c r="E24" s="22">
-        <v>-8457</v>
-      </c>
-      <c r="F24" s="23" t="str">
-        <v>-33.81%</v>
+        <v>28201</v>
+      </c>
+      <c r="E24" s="13">
+        <v>31652</v>
+      </c>
+      <c r="F24" s="14" t="str">
+        <v>52.88%</v>
       </c>
       <c r="G24" s="11" t="str">
         <v/>
@@ -1848,19 +1731,19 @@
         <v/>
       </c>
       <c r="B25" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Marketing</v>
       </c>
       <c r="C25" s="18">
-        <v>93369</v>
+        <v>67585</v>
       </c>
       <c r="D25" s="18">
-        <v>29468</v>
-      </c>
-      <c r="E25" s="24">
-        <v>63901</v>
-      </c>
-      <c r="F25" s="25" t="str">
-        <v>68.44%</v>
+        <v>38201</v>
+      </c>
+      <c r="E25" s="19">
+        <v>29384</v>
+      </c>
+      <c r="F25" s="20" t="str">
+        <v>43.48%</v>
       </c>
       <c r="G25" s="17" t="str">
         <v/>
@@ -1877,34 +1760,34 @@
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="str">
-        <v>2023-10</v>
+        <v>2023-07</v>
       </c>
       <c r="B26" s="5" t="str">
-        <v>Customer Support</v>
+        <v>Sales</v>
       </c>
       <c r="C26" s="6">
-        <v>13238</v>
+        <v>81835</v>
       </c>
       <c r="D26" s="6">
-        <v>37861</v>
-      </c>
-      <c r="E26" s="26">
-        <v>-24623</v>
-      </c>
-      <c r="F26" s="27" t="str">
-        <v>-186%</v>
+        <v>19697</v>
+      </c>
+      <c r="E26" s="7">
+        <v>62138</v>
+      </c>
+      <c r="F26" s="8" t="str">
+        <v>75.93%</v>
       </c>
       <c r="G26" s="6">
-        <v>38168</v>
+        <v>221898</v>
       </c>
       <c r="H26" s="6">
-        <v>115363</v>
-      </c>
-      <c r="I26" s="26">
-        <v>-77195</v>
-      </c>
-      <c r="J26" s="28">
-        <v>-207.06000000000003</v>
+        <v>68985</v>
+      </c>
+      <c r="I26" s="7">
+        <v>152913</v>
+      </c>
+      <c r="J26" s="9">
+        <v>58.343333333333334</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
@@ -1912,19 +1795,19 @@
         <v/>
       </c>
       <c r="B27" s="11" t="str">
-        <v>Marketing</v>
+        <v>Sales</v>
       </c>
       <c r="C27" s="12">
-        <v>14532</v>
+        <v>97703</v>
       </c>
       <c r="D27" s="12">
-        <v>40271</v>
-      </c>
-      <c r="E27" s="22">
-        <v>-25739</v>
-      </c>
-      <c r="F27" s="23" t="str">
-        <v>-177.12%</v>
+        <v>11552</v>
+      </c>
+      <c r="E27" s="13">
+        <v>86151</v>
+      </c>
+      <c r="F27" s="14" t="str">
+        <v>88.18%</v>
       </c>
       <c r="G27" s="11" t="str">
         <v/>
@@ -1944,19 +1827,19 @@
         <v/>
       </c>
       <c r="B28" s="17" t="str">
-        <v>Customer Support</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C28" s="18">
-        <v>10398</v>
+        <v>42360</v>
       </c>
       <c r="D28" s="18">
-        <v>37231</v>
+        <v>37736</v>
       </c>
       <c r="E28" s="19">
-        <v>-26833</v>
+        <v>4624</v>
       </c>
       <c r="F28" s="20" t="str">
-        <v>-258.06%</v>
+        <v>10.92%</v>
       </c>
       <c r="G28" s="17" t="str">
         <v/>
@@ -1973,34 +1856,34 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="str">
-        <v>2023-05</v>
+        <v>2023-07</v>
       </c>
       <c r="B29" s="5" t="str">
         <v>Customer Support</v>
       </c>
       <c r="C29" s="6">
-        <v>84822</v>
+        <v>84841</v>
       </c>
       <c r="D29" s="6">
-        <v>28335</v>
+        <v>46129</v>
       </c>
       <c r="E29" s="7">
-        <v>56487</v>
+        <v>38712</v>
       </c>
       <c r="F29" s="8" t="str">
-        <v>66.59%</v>
+        <v>45.63%</v>
       </c>
       <c r="G29" s="6">
-        <v>154584</v>
+        <v>210422</v>
       </c>
       <c r="H29" s="6">
-        <v>84333</v>
+        <v>100523</v>
       </c>
       <c r="I29" s="7">
-        <v>70251</v>
+        <v>109899</v>
       </c>
       <c r="J29" s="9">
-        <v>37.11333333333334</v>
+        <v>52.89000000000001</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
@@ -2008,19 +1891,19 @@
         <v/>
       </c>
       <c r="B30" s="11" t="str">
-        <v>R&amp;D</v>
+        <v>Human Resources</v>
       </c>
       <c r="C30" s="12">
-        <v>40004</v>
+        <v>79421</v>
       </c>
       <c r="D30" s="12">
-        <v>38266</v>
+        <v>34039</v>
       </c>
       <c r="E30" s="13">
-        <v>1738</v>
+        <v>45382</v>
       </c>
       <c r="F30" s="14" t="str">
-        <v>4.34%</v>
+        <v>57.14%</v>
       </c>
       <c r="G30" s="11" t="str">
         <v/>
@@ -2040,19 +1923,19 @@
         <v/>
       </c>
       <c r="B31" s="17" t="str">
-        <v>Human Resources</v>
+        <v>Sales</v>
       </c>
       <c r="C31" s="18">
-        <v>29758</v>
+        <v>46160</v>
       </c>
       <c r="D31" s="18">
-        <v>17732</v>
-      </c>
-      <c r="E31" s="24">
-        <v>12026</v>
-      </c>
-      <c r="F31" s="25" t="str">
-        <v>40.41%</v>
+        <v>20355</v>
+      </c>
+      <c r="E31" s="19">
+        <v>25805</v>
+      </c>
+      <c r="F31" s="20" t="str">
+        <v>55.9%</v>
       </c>
       <c r="G31" s="17" t="str">
         <v/>
@@ -2068,17 +1951,17 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="G32" s="29">
-        <v>1706015</v>
-      </c>
-      <c r="H32" s="29">
-        <v>887654</v>
-      </c>
-      <c r="I32" s="30">
-        <v>818361</v>
-      </c>
-      <c r="J32" s="31">
-        <v>17.074666666666666</v>
+      <c r="G32" s="24">
+        <v>1770989</v>
+      </c>
+      <c r="H32" s="24">
+        <v>906097</v>
+      </c>
+      <c r="I32" s="25">
+        <v>864892</v>
+      </c>
+      <c r="J32" s="26">
+        <v>41.82899999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: replace column "key" with "accessor"
</commit_message>
<xml_diff>
--- a/examples/financial-report.xlsx
+++ b/examples/financial-report.xlsx
@@ -32,7 +32,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="10">
+  <numFmts count="12">
     <numFmt numFmtId="165" formatCode="MMM YYYY"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
@@ -43,8 +43,10 @@
     <numFmt numFmtId="172" formatCode="$#,##0.00"/>
     <numFmt numFmtId="173" formatCode="$#,##0.00"/>
     <numFmt numFmtId="174" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="175" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -92,6 +94,31 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <color rgb="007500"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
     </font>
     <font>
       <sz val="11"/>
@@ -157,7 +184,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -464,6 +491,36 @@
       <right style="thin">
         <color rgb="000000"/>
       </right>
+      <top style="medium">
+        <color rgb="000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="000000"/>
+      </right>
       <top style="thin">
         <color rgb="000000"/>
       </top>
@@ -483,6 +540,51 @@
         <color rgb="000000"/>
       </top>
       <bottom style="medium">
+        <color rgb="000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="000000"/>
+      </top>
+      <bottom style="thin">
         <color rgb="000000"/>
       </bottom>
       <diagonal/>
@@ -536,7 +638,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -603,13 +705,28 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="13" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="14" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="17" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="18" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -992,34 +1109,34 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="4" t="str">
-        <v>2023-10</v>
+        <v>2023-05</v>
       </c>
       <c r="B2" s="5" t="str">
-        <v>Customer Support</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C2" s="6">
-        <v>75123</v>
+        <v>98402</v>
       </c>
       <c r="D2" s="6">
-        <v>20926</v>
+        <v>48363</v>
       </c>
       <c r="E2" s="7">
-        <v>54197</v>
+        <v>50039</v>
       </c>
       <c r="F2" s="8" t="str">
-        <v>72.14%</v>
+        <v>50.85%</v>
       </c>
       <c r="G2" s="6">
-        <v>158871</v>
+        <v>214285</v>
       </c>
       <c r="H2" s="6">
-        <v>86095</v>
+        <v>81907</v>
       </c>
       <c r="I2" s="7">
-        <v>72776</v>
+        <v>132378</v>
       </c>
       <c r="J2" s="9">
-        <v>37.83</v>
+        <v>64.37</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -1027,19 +1144,19 @@
         <v/>
       </c>
       <c r="B3" s="11" t="str">
-        <v>Customer Support</v>
+        <v>Human Resources</v>
       </c>
       <c r="C3" s="12">
-        <v>20752</v>
+        <v>57522</v>
       </c>
       <c r="D3" s="12">
-        <v>17084</v>
+        <v>10485</v>
       </c>
       <c r="E3" s="13">
-        <v>3668</v>
+        <v>47037</v>
       </c>
       <c r="F3" s="14" t="str">
-        <v>17.68%</v>
+        <v>81.77%</v>
       </c>
       <c r="G3" s="11" t="str">
         <v/>
@@ -1059,19 +1176,19 @@
         <v/>
       </c>
       <c r="B4" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="C4" s="18">
-        <v>62996</v>
+        <v>58361</v>
       </c>
       <c r="D4" s="18">
-        <v>48085</v>
+        <v>23059</v>
       </c>
       <c r="E4" s="19">
-        <v>14911</v>
+        <v>35302</v>
       </c>
       <c r="F4" s="20" t="str">
-        <v>23.67%</v>
+        <v>60.49%</v>
       </c>
       <c r="G4" s="17" t="str">
         <v/>
@@ -1088,34 +1205,34 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="str">
-        <v>2023-03</v>
+        <v>2023-01</v>
       </c>
       <c r="B5" s="5" t="str">
-        <v>Human Resources</v>
+        <v>Marketing</v>
       </c>
       <c r="C5" s="6">
-        <v>42667</v>
+        <v>37880</v>
       </c>
       <c r="D5" s="6">
-        <v>10024</v>
+        <v>16718</v>
       </c>
       <c r="E5" s="7">
-        <v>32643</v>
+        <v>21162</v>
       </c>
       <c r="F5" s="8" t="str">
-        <v>76.51%</v>
+        <v>55.87%</v>
       </c>
       <c r="G5" s="6">
-        <v>143580</v>
+        <v>147287</v>
       </c>
       <c r="H5" s="6">
-        <v>94408</v>
+        <v>61429</v>
       </c>
       <c r="I5" s="7">
-        <v>49172</v>
+        <v>85858</v>
       </c>
       <c r="J5" s="9">
-        <v>35.513333333333335</v>
+        <v>54.90333333333333</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -1123,19 +1240,19 @@
         <v/>
       </c>
       <c r="B6" s="11" t="str">
-        <v>Sales</v>
+        <v>Marketing</v>
       </c>
       <c r="C6" s="12">
-        <v>56344</v>
+        <v>21957</v>
       </c>
       <c r="D6" s="12">
-        <v>41280</v>
+        <v>11738</v>
       </c>
       <c r="E6" s="13">
-        <v>15064</v>
+        <v>10219</v>
       </c>
       <c r="F6" s="14" t="str">
-        <v>26.74%</v>
+        <v>46.54%</v>
       </c>
       <c r="G6" s="11" t="str">
         <v/>
@@ -1155,19 +1272,19 @@
         <v/>
       </c>
       <c r="B7" s="17" t="str">
-        <v>Human Resources</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C7" s="18">
-        <v>44569</v>
+        <v>87450</v>
       </c>
       <c r="D7" s="18">
-        <v>43104</v>
+        <v>32973</v>
       </c>
       <c r="E7" s="19">
-        <v>1465</v>
+        <v>54477</v>
       </c>
       <c r="F7" s="20" t="str">
-        <v>3.29%</v>
+        <v>62.3%</v>
       </c>
       <c r="G7" s="17" t="str">
         <v/>
@@ -1184,34 +1301,34 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="str">
-        <v>2023-06</v>
+        <v>2023-04</v>
       </c>
       <c r="B8" s="5" t="str">
-        <v>Human Resources</v>
+        <v>Customer Support</v>
       </c>
       <c r="C8" s="6">
-        <v>59635</v>
+        <v>87027</v>
       </c>
       <c r="D8" s="6">
-        <v>25739</v>
+        <v>33839</v>
       </c>
       <c r="E8" s="7">
-        <v>33896</v>
+        <v>53188</v>
       </c>
       <c r="F8" s="8" t="str">
-        <v>56.84%</v>
+        <v>61.12%</v>
       </c>
       <c r="G8" s="6">
-        <v>252115</v>
+        <v>206117</v>
       </c>
       <c r="H8" s="6">
-        <v>117520</v>
+        <v>106566</v>
       </c>
       <c r="I8" s="7">
-        <v>134595</v>
+        <v>99551</v>
       </c>
       <c r="J8" s="9">
-        <v>53.75333333333333</v>
+        <v>46.339999999999996</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -1219,19 +1336,19 @@
         <v/>
       </c>
       <c r="B9" s="11" t="str">
-        <v>Sales</v>
+        <v>Marketing</v>
       </c>
       <c r="C9" s="12">
-        <v>93467</v>
+        <v>58814</v>
       </c>
       <c r="D9" s="12">
-        <v>48184</v>
+        <v>34990</v>
       </c>
       <c r="E9" s="13">
-        <v>45283</v>
+        <v>23824</v>
       </c>
       <c r="F9" s="14" t="str">
-        <v>48.45%</v>
+        <v>40.51%</v>
       </c>
       <c r="G9" s="11" t="str">
         <v/>
@@ -1251,19 +1368,19 @@
         <v/>
       </c>
       <c r="B10" s="17" t="str">
-        <v>Sales</v>
+        <v>Marketing</v>
       </c>
       <c r="C10" s="18">
-        <v>99013</v>
+        <v>60276</v>
       </c>
       <c r="D10" s="18">
-        <v>43597</v>
+        <v>37737</v>
       </c>
       <c r="E10" s="19">
-        <v>55416</v>
+        <v>22539</v>
       </c>
       <c r="F10" s="20" t="str">
-        <v>55.97%</v>
+        <v>37.39%</v>
       </c>
       <c r="G10" s="17" t="str">
         <v/>
@@ -1280,34 +1397,34 @@
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="str">
-        <v>2023-12</v>
+        <v>2023-01</v>
       </c>
       <c r="B11" s="5" t="str">
-        <v>Human Resources</v>
+        <v>Sales</v>
       </c>
       <c r="C11" s="6">
-        <v>69443</v>
+        <v>29318</v>
       </c>
       <c r="D11" s="6">
-        <v>43038</v>
-      </c>
-      <c r="E11" s="7">
-        <v>26405</v>
-      </c>
-      <c r="F11" s="8" t="str">
-        <v>38.02%</v>
+        <v>43172</v>
+      </c>
+      <c r="E11" s="22">
+        <v>-13854</v>
+      </c>
+      <c r="F11" s="23" t="str">
+        <v>-47.25%</v>
       </c>
       <c r="G11" s="6">
-        <v>153944</v>
+        <v>171427</v>
       </c>
       <c r="H11" s="6">
-        <v>83220</v>
+        <v>107948</v>
       </c>
       <c r="I11" s="7">
-        <v>70724</v>
+        <v>63479</v>
       </c>
       <c r="J11" s="9">
-        <v>34.59</v>
+        <v>20.913333333333334</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -1315,19 +1432,19 @@
         <v/>
       </c>
       <c r="B12" s="11" t="str">
-        <v>Sales</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C12" s="12">
-        <v>62410</v>
+        <v>84867</v>
       </c>
       <c r="D12" s="12">
-        <v>16290</v>
+        <v>40704</v>
       </c>
       <c r="E12" s="13">
-        <v>46120</v>
+        <v>44163</v>
       </c>
       <c r="F12" s="14" t="str">
-        <v>73.9%</v>
+        <v>52.04%</v>
       </c>
       <c r="G12" s="11" t="str">
         <v/>
@@ -1347,19 +1464,19 @@
         <v/>
       </c>
       <c r="B13" s="17" t="str">
-        <v>Marketing</v>
+        <v>Human Resources</v>
       </c>
       <c r="C13" s="18">
-        <v>22091</v>
+        <v>57242</v>
       </c>
       <c r="D13" s="18">
-        <v>23892</v>
-      </c>
-      <c r="E13" s="22">
-        <v>-1801</v>
-      </c>
-      <c r="F13" s="23" t="str">
-        <v>-8.15%</v>
+        <v>24072</v>
+      </c>
+      <c r="E13" s="19">
+        <v>33170</v>
+      </c>
+      <c r="F13" s="20" t="str">
+        <v>57.95%</v>
       </c>
       <c r="G13" s="17" t="str">
         <v/>
@@ -1376,34 +1493,34 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="str">
-        <v>2023-03</v>
+        <v>2023-04</v>
       </c>
       <c r="B14" s="5" t="str">
-        <v>Marketing</v>
+        <v>Sales</v>
       </c>
       <c r="C14" s="6">
-        <v>58907</v>
+        <v>45492</v>
       </c>
       <c r="D14" s="6">
-        <v>14681</v>
+        <v>42419</v>
       </c>
       <c r="E14" s="7">
-        <v>44226</v>
+        <v>3073</v>
       </c>
       <c r="F14" s="8" t="str">
-        <v>75.08%</v>
+        <v>6.76%</v>
       </c>
       <c r="G14" s="6">
-        <v>105805</v>
+        <v>134048</v>
       </c>
       <c r="H14" s="6">
-        <v>47122</v>
+        <v>85718</v>
       </c>
       <c r="I14" s="7">
-        <v>58683</v>
+        <v>48330</v>
       </c>
       <c r="J14" s="9">
-        <v>44.96333333333333</v>
+        <v>5.940000000000002</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -1411,19 +1528,19 @@
         <v/>
       </c>
       <c r="B15" s="11" t="str">
-        <v>Customer Support</v>
+        <v>Sales</v>
       </c>
       <c r="C15" s="12">
-        <v>24859</v>
+        <v>72852</v>
       </c>
       <c r="D15" s="12">
-        <v>13627</v>
+        <v>17373</v>
       </c>
       <c r="E15" s="13">
-        <v>11232</v>
+        <v>55479</v>
       </c>
       <c r="F15" s="14" t="str">
-        <v>45.18%</v>
+        <v>76.15%</v>
       </c>
       <c r="G15" s="11" t="str">
         <v/>
@@ -1443,19 +1560,19 @@
         <v/>
       </c>
       <c r="B16" s="17" t="str">
-        <v>Customer Support</v>
+        <v>Human Resources</v>
       </c>
       <c r="C16" s="18">
-        <v>22039</v>
+        <v>15704</v>
       </c>
       <c r="D16" s="18">
-        <v>18814</v>
-      </c>
-      <c r="E16" s="19">
-        <v>3225</v>
-      </c>
-      <c r="F16" s="20" t="str">
-        <v>14.63%</v>
+        <v>25926</v>
+      </c>
+      <c r="E16" s="24">
+        <v>-10222</v>
+      </c>
+      <c r="F16" s="25" t="str">
+        <v>-65.09%</v>
       </c>
       <c r="G16" s="17" t="str">
         <v/>
@@ -1472,34 +1589,34 @@
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="str">
-        <v>2023-12</v>
+        <v>2023-06</v>
       </c>
       <c r="B17" s="5" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="C17" s="6">
-        <v>75289</v>
+        <v>94774</v>
       </c>
       <c r="D17" s="6">
-        <v>39784</v>
+        <v>30906</v>
       </c>
       <c r="E17" s="7">
-        <v>35505</v>
+        <v>63868</v>
       </c>
       <c r="F17" s="8" t="str">
-        <v>47.16%</v>
+        <v>67.39%</v>
       </c>
       <c r="G17" s="6">
-        <v>161258</v>
+        <v>283722</v>
       </c>
       <c r="H17" s="6">
-        <v>118258</v>
+        <v>69954</v>
       </c>
       <c r="I17" s="7">
-        <v>43000</v>
+        <v>213768</v>
       </c>
       <c r="J17" s="9">
-        <v>15.86</v>
+        <v>75.16</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -1507,19 +1624,19 @@
         <v/>
       </c>
       <c r="B18" s="11" t="str">
-        <v>Customer Support</v>
+        <v>Sales</v>
       </c>
       <c r="C18" s="12">
-        <v>58928</v>
+        <v>90291</v>
       </c>
       <c r="D18" s="12">
-        <v>45290</v>
+        <v>24896</v>
       </c>
       <c r="E18" s="13">
-        <v>13638</v>
+        <v>65395</v>
       </c>
       <c r="F18" s="14" t="str">
-        <v>23.14%</v>
+        <v>72.43%</v>
       </c>
       <c r="G18" s="11" t="str">
         <v/>
@@ -1539,19 +1656,19 @@
         <v/>
       </c>
       <c r="B19" s="17" t="str">
-        <v>Marketing</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C19" s="18">
-        <v>27041</v>
+        <v>98657</v>
       </c>
       <c r="D19" s="18">
-        <v>33184</v>
-      </c>
-      <c r="E19" s="22">
-        <v>-6143</v>
-      </c>
-      <c r="F19" s="23" t="str">
-        <v>-22.72%</v>
+        <v>14152</v>
+      </c>
+      <c r="E19" s="19">
+        <v>84505</v>
+      </c>
+      <c r="F19" s="20" t="str">
+        <v>85.66%</v>
       </c>
       <c r="G19" s="17" t="str">
         <v/>
@@ -1568,34 +1685,34 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="str">
-        <v>2023-07</v>
+        <v>2023-05</v>
       </c>
       <c r="B20" s="5" t="str">
         <v>Sales</v>
       </c>
       <c r="C20" s="6">
-        <v>40407</v>
+        <v>41056</v>
       </c>
       <c r="D20" s="6">
-        <v>31604</v>
-      </c>
-      <c r="E20" s="7">
-        <v>8803</v>
-      </c>
-      <c r="F20" s="8" t="str">
-        <v>21.79%</v>
+        <v>43370</v>
+      </c>
+      <c r="E20" s="22">
+        <v>-2314</v>
+      </c>
+      <c r="F20" s="23" t="str">
+        <v>-5.64%</v>
       </c>
       <c r="G20" s="6">
-        <v>196964</v>
+        <v>85456</v>
       </c>
       <c r="H20" s="6">
-        <v>88282</v>
+        <v>66952</v>
       </c>
       <c r="I20" s="7">
-        <v>108682</v>
+        <v>18504</v>
       </c>
       <c r="J20" s="9">
-        <v>49.48666666666666</v>
+        <v>29.833333333333332</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1603,19 +1720,19 @@
         <v/>
       </c>
       <c r="B21" s="11" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="C21" s="12">
-        <v>87221</v>
+        <v>25718</v>
       </c>
       <c r="D21" s="12">
-        <v>28428</v>
+        <v>14590</v>
       </c>
       <c r="E21" s="13">
-        <v>58793</v>
+        <v>11128</v>
       </c>
       <c r="F21" s="14" t="str">
-        <v>67.41%</v>
+        <v>43.27%</v>
       </c>
       <c r="G21" s="11" t="str">
         <v/>
@@ -1635,19 +1752,19 @@
         <v/>
       </c>
       <c r="B22" s="17" t="str">
-        <v>Human Resources</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C22" s="18">
-        <v>69336</v>
+        <v>18682</v>
       </c>
       <c r="D22" s="18">
-        <v>28250</v>
+        <v>8992</v>
       </c>
       <c r="E22" s="19">
-        <v>41086</v>
+        <v>9690</v>
       </c>
       <c r="F22" s="20" t="str">
-        <v>59.26%</v>
+        <v>51.87%</v>
       </c>
       <c r="G22" s="17" t="str">
         <v/>
@@ -1664,34 +1781,34 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="str">
-        <v>2023-08</v>
+        <v>2023-06</v>
       </c>
       <c r="B23" s="5" t="str">
-        <v>R&amp;D</v>
+        <v>Customer Support</v>
       </c>
       <c r="C23" s="6">
-        <v>38694</v>
+        <v>73610</v>
       </c>
       <c r="D23" s="6">
-        <v>35282</v>
+        <v>8514</v>
       </c>
       <c r="E23" s="7">
-        <v>3412</v>
+        <v>65096</v>
       </c>
       <c r="F23" s="8" t="str">
-        <v>8.82%</v>
+        <v>88.43%</v>
       </c>
       <c r="G23" s="6">
-        <v>166132</v>
+        <v>220991</v>
       </c>
       <c r="H23" s="6">
-        <v>101684</v>
+        <v>50730</v>
       </c>
       <c r="I23" s="7">
-        <v>64448</v>
+        <v>170261</v>
       </c>
       <c r="J23" s="9">
-        <v>35.06</v>
+        <v>77.32000000000001</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
@@ -1702,16 +1819,16 @@
         <v>Customer Support</v>
       </c>
       <c r="C24" s="12">
-        <v>59853</v>
+        <v>85337</v>
       </c>
       <c r="D24" s="12">
-        <v>28201</v>
+        <v>26296</v>
       </c>
       <c r="E24" s="13">
-        <v>31652</v>
+        <v>59041</v>
       </c>
       <c r="F24" s="14" t="str">
-        <v>52.88%</v>
+        <v>69.19%</v>
       </c>
       <c r="G24" s="11" t="str">
         <v/>
@@ -1731,19 +1848,19 @@
         <v/>
       </c>
       <c r="B25" s="17" t="str">
-        <v>Marketing</v>
+        <v>Human Resources</v>
       </c>
       <c r="C25" s="18">
-        <v>67585</v>
+        <v>62044</v>
       </c>
       <c r="D25" s="18">
-        <v>38201</v>
+        <v>15920</v>
       </c>
       <c r="E25" s="19">
-        <v>29384</v>
+        <v>46124</v>
       </c>
       <c r="F25" s="20" t="str">
-        <v>43.48%</v>
+        <v>74.34%</v>
       </c>
       <c r="G25" s="17" t="str">
         <v/>
@@ -1760,34 +1877,34 @@
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="str">
-        <v>2023-07</v>
+        <v>2023-10</v>
       </c>
       <c r="B26" s="5" t="str">
-        <v>Sales</v>
+        <v>R&amp;D</v>
       </c>
       <c r="C26" s="6">
-        <v>81835</v>
+        <v>55164</v>
       </c>
       <c r="D26" s="6">
-        <v>19697</v>
+        <v>5086</v>
       </c>
       <c r="E26" s="7">
-        <v>62138</v>
+        <v>50078</v>
       </c>
       <c r="F26" s="8" t="str">
-        <v>75.93%</v>
+        <v>90.78%</v>
       </c>
       <c r="G26" s="6">
-        <v>221898</v>
+        <v>241696</v>
       </c>
       <c r="H26" s="6">
-        <v>68985</v>
+        <v>52508</v>
       </c>
       <c r="I26" s="7">
-        <v>152913</v>
+        <v>189188</v>
       </c>
       <c r="J26" s="9">
-        <v>58.343333333333334</v>
+        <v>80.05</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
@@ -1795,19 +1912,19 @@
         <v/>
       </c>
       <c r="B27" s="11" t="str">
-        <v>Sales</v>
+        <v>Human Resources</v>
       </c>
       <c r="C27" s="12">
-        <v>97703</v>
+        <v>91747</v>
       </c>
       <c r="D27" s="12">
-        <v>11552</v>
+        <v>17053</v>
       </c>
       <c r="E27" s="13">
-        <v>86151</v>
+        <v>74694</v>
       </c>
       <c r="F27" s="14" t="str">
-        <v>88.18%</v>
+        <v>81.41%</v>
       </c>
       <c r="G27" s="11" t="str">
         <v/>
@@ -1827,19 +1944,19 @@
         <v/>
       </c>
       <c r="B28" s="17" t="str">
-        <v>R&amp;D</v>
+        <v>Marketing</v>
       </c>
       <c r="C28" s="18">
-        <v>42360</v>
+        <v>94785</v>
       </c>
       <c r="D28" s="18">
-        <v>37736</v>
+        <v>30369</v>
       </c>
       <c r="E28" s="19">
-        <v>4624</v>
+        <v>64416</v>
       </c>
       <c r="F28" s="20" t="str">
-        <v>10.92%</v>
+        <v>67.96%</v>
       </c>
       <c r="G28" s="17" t="str">
         <v/>
@@ -1856,34 +1973,34 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="str">
-        <v>2023-07</v>
+        <v>2023-11</v>
       </c>
       <c r="B29" s="5" t="str">
-        <v>Customer Support</v>
+        <v>Sales</v>
       </c>
       <c r="C29" s="6">
-        <v>84841</v>
+        <v>48721</v>
       </c>
       <c r="D29" s="6">
-        <v>46129</v>
-      </c>
-      <c r="E29" s="7">
-        <v>38712</v>
-      </c>
-      <c r="F29" s="8" t="str">
-        <v>45.63%</v>
+        <v>49409</v>
+      </c>
+      <c r="E29" s="22">
+        <v>-688</v>
+      </c>
+      <c r="F29" s="23" t="str">
+        <v>-1.41%</v>
       </c>
       <c r="G29" s="6">
-        <v>210422</v>
+        <v>108033</v>
       </c>
       <c r="H29" s="6">
-        <v>100523</v>
-      </c>
-      <c r="I29" s="7">
-        <v>109899</v>
-      </c>
-      <c r="J29" s="9">
-        <v>52.89000000000001</v>
+        <v>108599</v>
+      </c>
+      <c r="I29" s="22">
+        <v>-566</v>
+      </c>
+      <c r="J29" s="26">
+        <v>-5.293333333333334</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
@@ -1891,19 +2008,19 @@
         <v/>
       </c>
       <c r="B30" s="11" t="str">
-        <v>Human Resources</v>
+        <v>Marketing</v>
       </c>
       <c r="C30" s="12">
-        <v>79421</v>
+        <v>24159</v>
       </c>
       <c r="D30" s="12">
-        <v>34039</v>
-      </c>
-      <c r="E30" s="13">
-        <v>45382</v>
-      </c>
-      <c r="F30" s="14" t="str">
-        <v>57.14%</v>
+        <v>35606</v>
+      </c>
+      <c r="E30" s="27">
+        <v>-11447</v>
+      </c>
+      <c r="F30" s="28" t="str">
+        <v>-47.38%</v>
       </c>
       <c r="G30" s="11" t="str">
         <v/>
@@ -1923,19 +2040,19 @@
         <v/>
       </c>
       <c r="B31" s="17" t="str">
-        <v>Sales</v>
+        <v>Customer Support</v>
       </c>
       <c r="C31" s="18">
-        <v>46160</v>
+        <v>35153</v>
       </c>
       <c r="D31" s="18">
-        <v>20355</v>
+        <v>23584</v>
       </c>
       <c r="E31" s="19">
-        <v>25805</v>
+        <v>11569</v>
       </c>
       <c r="F31" s="20" t="str">
-        <v>55.9%</v>
+        <v>32.91%</v>
       </c>
       <c r="G31" s="17" t="str">
         <v/>
@@ -1951,17 +2068,17 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="G32" s="24">
-        <v>1770989</v>
-      </c>
-      <c r="H32" s="24">
-        <v>906097</v>
-      </c>
-      <c r="I32" s="25">
-        <v>864892</v>
-      </c>
-      <c r="J32" s="26">
-        <v>41.82899999999999</v>
+      <c r="G32" s="29">
+        <v>1813062</v>
+      </c>
+      <c r="H32" s="29">
+        <v>792311</v>
+      </c>
+      <c r="I32" s="30">
+        <v>1020751</v>
+      </c>
+      <c r="J32" s="31">
+        <v>44.95366666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>